<commit_message>
Finalize proposal assets and experience design
</commit_message>
<xml_diff>
--- a/public/commercial/quotation.xlsx
+++ b/public/commercial/quotation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohamed.akram.PARADIGM-EG\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D67B8CB-84C7-472F-B62E-1BAE7E35E86A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C0E4DD6-F89B-47F8-A887-F3793821DDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="148">
   <si>
     <t>PARADIGM CAPITAL GROUP</t>
   </si>
@@ -479,6 +479,10 @@
   </si>
   <si>
     <t>El Gouna · 10–12 Sep 2026 · ~500 delegates · EGP</t>
+  </si>
+  <si>
+    <t>Please note that if a testing day is required, an additional 50% will be applied to the Audio-Visual. Production and visibility 
+items will remain at the same cost</t>
   </si>
 </sst>
 </file>
@@ -489,7 +493,7 @@
     <numFmt numFmtId="164" formatCode="#,##0&quot; EGP&quot;;\-#,##0&quot; EGP&quot;;\—"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -654,6 +658,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -699,7 +710,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -759,11 +770,73 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC7D3E0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFC7D3E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFC7D3E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFC7D3E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFC7D3E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC7D3E0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFC7D3E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFC7D3E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFC7D3E0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFC7D3E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -809,65 +882,83 @@
     <xf numFmtId="164" fontId="18" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1188,7 +1279,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -1201,69 +1292,69 @@
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
-      <c r="B2" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="B2" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="32" t="s">
         <v>132</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="34" t="s">
         <v>146</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
     </row>
     <row r="6" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
     </row>
     <row r="7" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29"/>
     </row>
     <row r="8" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
@@ -1292,7 +1383,7 @@
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="20" t="s">
         <v>145</v>
       </c>
       <c r="C9" s="7" t="s">
@@ -1316,7 +1407,7 @@
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="20" t="s">
         <v>137</v>
       </c>
       <c r="C10" s="7" t="s">
@@ -1340,7 +1431,7 @@
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="20" t="s">
         <v>139</v>
       </c>
       <c r="C11" s="7" t="s">
@@ -1388,7 +1479,7 @@
       <c r="A13" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="20" t="s">
         <v>143</v>
       </c>
       <c r="C13" s="7" t="s">
@@ -1460,7 +1551,7 @@
       <c r="A16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="20" t="s">
         <v>138</v>
       </c>
       <c r="C16" s="7" t="s">
@@ -1577,29 +1668,29 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
       <c r="G21" s="10">
         <f>SUM(G9:G20)</f>
         <v>1186500</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
     </row>
     <row r="23" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
@@ -1628,7 +1719,7 @@
       <c r="A24" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="20" t="s">
         <v>144</v>
       </c>
       <c r="C24" s="7" t="s">
@@ -1700,7 +1791,7 @@
       <c r="A27" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="20" t="s">
         <v>140</v>
       </c>
       <c r="C27" s="7" t="s">
@@ -1803,7 +1894,7 @@
         <v>11</v>
       </c>
       <c r="D31" s="7">
-        <v>250</v>
+        <v>65</v>
       </c>
       <c r="E31" s="7">
         <v>1</v>
@@ -1813,7 +1904,7 @@
       </c>
       <c r="G31" s="9">
         <f t="shared" si="1"/>
-        <v>112500</v>
+        <v>29250</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1841,40 +1932,40 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="23" t="s">
+      <c r="A33" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="B33" s="23"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
       <c r="G33" s="10">
         <f>SUM(G24:G32)</f>
-        <v>712800</v>
+        <v>629550</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="21" t="s">
+      <c r="A34" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="21"/>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
     </row>
     <row r="35" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
     </row>
     <row r="36" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
@@ -1924,29 +2015,29 @@
       </c>
     </row>
     <row r="38" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="23" t="s">
+      <c r="A38" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="23"/>
-      <c r="F38" s="23"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="21"/>
       <c r="G38" s="10">
         <f>SUM(G37:G37)</f>
         <v>26000</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="B39" s="21"/>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
     </row>
     <row r="40" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
@@ -2092,40 +2183,40 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="23" t="s">
+      <c r="A46" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="B46" s="23"/>
-      <c r="C46" s="23"/>
-      <c r="D46" s="23"/>
-      <c r="E46" s="23"/>
-      <c r="F46" s="23"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
       <c r="G46" s="10">
         <f>SUM(G41:G45)</f>
         <v>249000</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="21" t="s">
+      <c r="A47" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="B47" s="21"/>
-      <c r="C47" s="21"/>
-      <c r="D47" s="21"/>
-      <c r="E47" s="21"/>
-      <c r="F47" s="21"/>
-      <c r="G47" s="21"/>
+      <c r="B47" s="23"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="22" t="s">
+      <c r="A48" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="B48" s="22"/>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="22"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
     </row>
     <row r="49" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
@@ -2175,13 +2266,13 @@
       </c>
     </row>
     <row r="51" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="27" t="s">
+      <c r="A51" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="B51" s="29" t="s">
+      <c r="B51" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="C51" s="28" t="s">
+      <c r="C51" s="19" t="s">
         <v>5</v>
       </c>
       <c r="D51" s="7">
@@ -2247,42 +2338,42 @@
       </c>
     </row>
     <row r="54" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="31" t="s">
+      <c r="A54" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="B54" s="23"/>
-      <c r="C54" s="23"/>
-      <c r="D54" s="23"/>
-      <c r="E54" s="23"/>
-      <c r="F54" s="23"/>
+      <c r="B54" s="21"/>
+      <c r="C54" s="21"/>
+      <c r="D54" s="21"/>
+      <c r="E54" s="21"/>
+      <c r="F54" s="21"/>
       <c r="G54" s="10">
         <f>SUM(G50:G53)</f>
         <v>508000</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="21" t="s">
+      <c r="A55" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="B55" s="21"/>
-      <c r="C55" s="21"/>
-      <c r="D55" s="21"/>
-      <c r="E55" s="21"/>
-      <c r="F55" s="21"/>
-      <c r="G55" s="21"/>
+      <c r="B55" s="23"/>
+      <c r="C55" s="23"/>
+      <c r="D55" s="23"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="23"/>
     </row>
     <row r="56" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="24" t="s">
+      <c r="A56" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="B56" s="24"/>
-      <c r="C56" s="24"/>
-      <c r="D56" s="24"/>
-      <c r="E56" s="24"/>
-      <c r="F56" s="24"/>
+      <c r="B56" s="28"/>
+      <c r="C56" s="28"/>
+      <c r="D56" s="28"/>
+      <c r="E56" s="28"/>
+      <c r="F56" s="28"/>
       <c r="G56" s="12">
         <f>SUM(G21,G33,G38,G46,G54)</f>
-        <v>2682300</v>
+        <v>2599050</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
@@ -2312,586 +2403,610 @@
       <c r="G58" s="11"/>
     </row>
     <row r="59" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="25" t="s">
+      <c r="A59" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="B59" s="25"/>
-      <c r="C59" s="25"/>
-      <c r="D59" s="25"/>
-      <c r="E59" s="25"/>
-      <c r="F59" s="25"/>
+      <c r="B59" s="22"/>
+      <c r="C59" s="22"/>
+      <c r="D59" s="22"/>
+      <c r="E59" s="22"/>
+      <c r="F59" s="22"/>
       <c r="G59" s="15">
         <f>G56*$B$57</f>
-        <v>402345</v>
+        <v>389857.5</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="25" t="s">
+      <c r="A60" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="B60" s="25"/>
-      <c r="C60" s="25"/>
-      <c r="D60" s="25"/>
-      <c r="E60" s="25"/>
-      <c r="F60" s="25"/>
+      <c r="B60" s="22"/>
+      <c r="C60" s="22"/>
+      <c r="D60" s="22"/>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
       <c r="G60" s="15">
         <f>G56+G59</f>
-        <v>3084645</v>
+        <v>2988907.5</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="25" t="s">
+      <c r="A61" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="B61" s="25"/>
-      <c r="C61" s="25"/>
-      <c r="D61" s="25"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="25"/>
+      <c r="B61" s="22"/>
+      <c r="C61" s="22"/>
+      <c r="D61" s="22"/>
+      <c r="E61" s="22"/>
+      <c r="F61" s="22"/>
       <c r="G61" s="15">
         <f>G60*$B$58</f>
-        <v>431850.30000000005</v>
+        <v>418447.05000000005</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="32" t="s">
+      <c r="A62" s="42" t="s">
         <v>102</v>
       </c>
-      <c r="B62" s="32"/>
-      <c r="C62" s="32"/>
-      <c r="D62" s="32"/>
-      <c r="E62" s="32"/>
-      <c r="F62" s="32"/>
+      <c r="B62" s="42"/>
+      <c r="C62" s="42"/>
+      <c r="D62" s="42"/>
+      <c r="E62" s="42"/>
+      <c r="F62" s="42"/>
       <c r="G62" s="16">
         <f>G60+G61</f>
-        <v>3516495.3</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="33"/>
-      <c r="B63" s="34"/>
-      <c r="C63" s="34"/>
-      <c r="D63" s="34"/>
-      <c r="E63" s="34"/>
-      <c r="F63" s="34"/>
-      <c r="G63" s="35"/>
-    </row>
-    <row r="64" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="21" t="s">
+        <v>3407354.55</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="B63" s="37"/>
+      <c r="C63" s="37"/>
+      <c r="D63" s="37"/>
+      <c r="E63" s="37"/>
+      <c r="F63" s="37"/>
+      <c r="G63" s="38"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" s="39"/>
+      <c r="B64" s="40"/>
+      <c r="C64" s="40"/>
+      <c r="D64" s="40"/>
+      <c r="E64" s="40"/>
+      <c r="F64" s="40"/>
+      <c r="G64" s="41"/>
+    </row>
+    <row r="65" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="25"/>
+      <c r="B65" s="26"/>
+      <c r="C65" s="26"/>
+      <c r="D65" s="26"/>
+      <c r="E65" s="26"/>
+      <c r="F65" s="26"/>
+      <c r="G65" s="27"/>
+    </row>
+    <row r="66" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="B64" s="21"/>
-      <c r="C64" s="21"/>
-      <c r="D64" s="21"/>
-      <c r="E64" s="21"/>
-      <c r="F64" s="21"/>
-      <c r="G64" s="21"/>
-    </row>
-    <row r="65" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B65" s="2" t="s">
+      <c r="B66" s="23"/>
+      <c r="C66" s="23"/>
+      <c r="D66" s="23"/>
+      <c r="E66" s="23"/>
+      <c r="F66" s="23"/>
+      <c r="G66" s="23"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C67" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D65" s="3" t="s">
+      <c r="D67" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="E67" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F65" s="4" t="s">
+      <c r="F67" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G65" s="4" t="s">
+      <c r="G67" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="33" x14ac:dyDescent="0.35">
-      <c r="A66" s="5" t="s">
+    <row r="68" spans="1:7" ht="33" x14ac:dyDescent="0.35">
+      <c r="A68" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B66" s="29" t="s">
+      <c r="B68" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="C68" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="D66" s="26">
+      <c r="D68" s="17">
         <v>300</v>
       </c>
-      <c r="E66" s="26">
-        <v>1</v>
-      </c>
-      <c r="F66" s="8">
+      <c r="E68" s="17">
+        <v>1</v>
+      </c>
+      <c r="F68" s="8">
         <v>2500</v>
       </c>
-      <c r="G66" s="9">
-        <f>IF(OR(D66="",F66=""),0,D66*IF(E66="",1,E66)*F66)</f>
+      <c r="G68" s="9">
+        <f>IF(OR(D68="",F68=""),0,D68*IF(E68="",1,E68)*F68)</f>
         <v>750000</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="5" t="s">
+    <row r="69" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B67" s="6" t="s">
+      <c r="B69" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="C69" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D67" s="7">
-        <v>1</v>
-      </c>
-      <c r="E67" s="7">
-        <v>3</v>
-      </c>
-      <c r="F67" s="8">
+      <c r="D69" s="7">
+        <v>1</v>
+      </c>
+      <c r="E69" s="7">
+        <v>3</v>
+      </c>
+      <c r="F69" s="8">
         <v>6000</v>
       </c>
-      <c r="G67" s="9">
-        <f t="shared" ref="G67" si="3">IF(OR(D67="",F67=""),0,D67*IF(E67="",1,E67)*F67)</f>
+      <c r="G69" s="9">
+        <f t="shared" ref="G69" si="3">IF(OR(D69="",F69=""),0,D69*IF(E69="",1,E69)*F69)</f>
         <v>18000</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="27" t="s">
+    <row r="70" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A70" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="B68" s="29" t="s">
+      <c r="B70" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="C68" s="28" t="s">
+      <c r="C70" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="D68" s="26">
-        <v>1</v>
-      </c>
-      <c r="E68" s="26">
-        <v>1</v>
-      </c>
-      <c r="F68" s="8">
+      <c r="D70" s="17">
+        <v>1</v>
+      </c>
+      <c r="E70" s="17">
+        <v>1</v>
+      </c>
+      <c r="F70" s="8">
         <v>55000</v>
       </c>
-      <c r="G68" s="9">
-        <f t="shared" ref="G68:G71" si="4">IF(OR(D68="",F68=""),0,D68*IF(E68="",1,E68)*F68)</f>
+      <c r="G70" s="9">
+        <f t="shared" ref="G70:G73" si="4">IF(OR(D70="",F70=""),0,D70*IF(E70="",1,E70)*F70)</f>
         <v>55000</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="27" t="s">
+    <row r="71" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="B69" s="29" t="s">
+      <c r="B71" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="C69" s="28" t="s">
+      <c r="C71" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="D69" s="26">
-        <v>1</v>
-      </c>
-      <c r="E69" s="26">
-        <v>1</v>
-      </c>
-      <c r="F69" s="8">
+      <c r="D71" s="17">
+        <v>1</v>
+      </c>
+      <c r="E71" s="17">
+        <v>1</v>
+      </c>
+      <c r="F71" s="8">
         <v>150000</v>
       </c>
-      <c r="G69" s="9">
+      <c r="G71" s="9">
         <f t="shared" si="4"/>
         <v>150000</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="27" t="s">
+    <row r="72" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="B70" s="29" t="s">
+      <c r="B72" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="C70" s="28" t="s">
+      <c r="C72" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="D70" s="26">
-        <v>1</v>
-      </c>
-      <c r="E70" s="26">
-        <v>1</v>
-      </c>
-      <c r="F70" s="8">
+      <c r="D72" s="17">
+        <v>1</v>
+      </c>
+      <c r="E72" s="17">
+        <v>1</v>
+      </c>
+      <c r="F72" s="8">
         <v>80000</v>
       </c>
-      <c r="G70" s="9">
+      <c r="G72" s="9">
         <f t="shared" si="4"/>
         <v>80000</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="5" t="s">
+    <row r="73" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B71" s="6" t="s">
+      <c r="B73" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C71" s="7" t="s">
+      <c r="C73" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D71" s="7">
+      <c r="D73" s="7">
         <v>30</v>
       </c>
-      <c r="E71" s="7">
-        <v>1</v>
-      </c>
-      <c r="F71" s="8">
+      <c r="E73" s="7">
+        <v>1</v>
+      </c>
+      <c r="F73" s="8">
         <v>1000</v>
       </c>
-      <c r="G71" s="9">
+      <c r="G73" s="9">
         <f t="shared" si="4"/>
         <v>30000</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B72" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C72" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D72" s="7">
-        <v>2</v>
-      </c>
-      <c r="E72" s="7">
-        <v>3</v>
-      </c>
-      <c r="F72" s="8">
-        <v>3000</v>
-      </c>
-      <c r="G72" s="9">
-        <f>IF(OR(D72="",F72=""),0,D72*IF(E72="",1,E72)*F72)</f>
-        <v>18000</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B73" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C73" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D73" s="7">
-        <v>1</v>
-      </c>
-      <c r="E73" s="7">
-        <v>1</v>
-      </c>
-      <c r="F73" s="8">
-        <v>64000</v>
-      </c>
-      <c r="G73" s="9">
-        <f t="shared" ref="G73:G76" si="5">IF(OR(D73="",F73=""),0,D73*IF(E73="",1,E73)*F73)</f>
-        <v>64000</v>
-      </c>
-    </row>
     <row r="74" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D74" s="7">
+        <v>2</v>
+      </c>
+      <c r="E74" s="7">
+        <v>3</v>
+      </c>
+      <c r="F74" s="8">
+        <v>3000</v>
+      </c>
+      <c r="G74" s="9">
+        <f>IF(OR(D74="",F74=""),0,D74*IF(E74="",1,E74)*F74)</f>
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A75" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D75" s="7">
+        <v>1</v>
+      </c>
+      <c r="E75" s="7">
+        <v>1</v>
+      </c>
+      <c r="F75" s="8">
+        <v>64000</v>
+      </c>
+      <c r="G75" s="9">
+        <f t="shared" ref="G75:G79" si="5">IF(OR(D75="",F75=""),0,D75*IF(E75="",1,E75)*F75)</f>
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B74" s="6" t="s">
+      <c r="B76" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C74" s="7" t="s">
+      <c r="C76" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D74" s="7">
-        <v>1</v>
-      </c>
-      <c r="E74" s="7">
-        <v>1</v>
-      </c>
-      <c r="F74" s="8">
+      <c r="D76" s="7">
+        <v>1</v>
+      </c>
+      <c r="E76" s="7">
+        <v>1</v>
+      </c>
+      <c r="F76" s="8">
         <v>55000</v>
       </c>
-      <c r="G74" s="9">
+      <c r="G76" s="9">
         <f t="shared" si="5"/>
         <v>55000</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="5" t="s">
+    <row r="77" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A77" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B75" s="29" t="s">
+      <c r="B77" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="C75" s="7" t="s">
+      <c r="C77" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D75" s="7">
+      <c r="D77" s="7">
         <v>150</v>
       </c>
-      <c r="E75" s="7">
-        <v>1</v>
-      </c>
-      <c r="F75" s="8">
+      <c r="E77" s="7">
+        <v>1</v>
+      </c>
+      <c r="F77" s="8">
         <v>150</v>
       </c>
-      <c r="G75" s="9">
+      <c r="G77" s="9">
         <f t="shared" si="5"/>
         <v>22500</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="5" t="s">
+    <row r="78" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A78" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D78" s="7">
+        <v>65</v>
+      </c>
+      <c r="E78" s="7">
+        <v>1</v>
+      </c>
+      <c r="F78" s="8">
+        <v>450</v>
+      </c>
+      <c r="G78" s="9">
+        <f t="shared" si="5"/>
+        <v>29250</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A79" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B76" s="6" t="s">
+      <c r="B79" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C76" s="7" t="s">
+      <c r="C79" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D76" s="7">
-        <v>1</v>
-      </c>
-      <c r="E76" s="7">
-        <v>1</v>
-      </c>
-      <c r="F76" s="8">
+      <c r="D79" s="7">
+        <v>1</v>
+      </c>
+      <c r="E79" s="7">
+        <v>1</v>
+      </c>
+      <c r="F79" s="8">
         <v>40000</v>
       </c>
-      <c r="G76" s="9">
+      <c r="G79" s="9">
         <f t="shared" si="5"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="77" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="5" t="s">
+    <row r="80" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A80" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B77" s="6" t="s">
+      <c r="B80" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C77" s="7" t="s">
+      <c r="C80" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D77" s="7">
+      <c r="D80" s="7">
         <v>8</v>
       </c>
-      <c r="E77" s="7">
-        <v>3</v>
-      </c>
-      <c r="F77" s="8">
+      <c r="E80" s="7">
+        <v>3</v>
+      </c>
+      <c r="F80" s="8">
         <v>4500</v>
       </c>
-      <c r="G77" s="9">
-        <f t="shared" ref="G77:G78" si="6">IF(OR(D77="",F77=""),0,D77*IF(E77="",1,E77)*F77)</f>
+      <c r="G80" s="9">
+        <f t="shared" ref="G80:G81" si="6">IF(OR(D80="",F80=""),0,D80*IF(E80="",1,E80)*F80)</f>
         <v>108000</v>
       </c>
     </row>
-    <row r="78" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="5" t="s">
+    <row r="81" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A81" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B78" s="6" t="s">
+      <c r="B81" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C78" s="7" t="s">
+      <c r="C81" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D78" s="7">
-        <v>1</v>
-      </c>
-      <c r="E78" s="7">
-        <v>3</v>
-      </c>
-      <c r="F78" s="8">
+      <c r="D81" s="7">
+        <v>1</v>
+      </c>
+      <c r="E81" s="7">
+        <v>3</v>
+      </c>
+      <c r="F81" s="8">
         <v>20000</v>
       </c>
-      <c r="G78" s="9">
+      <c r="G81" s="9">
         <f t="shared" si="6"/>
         <v>60000</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="31" t="s">
+    <row r="82" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A82" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="B79" s="23"/>
-      <c r="C79" s="23"/>
-      <c r="D79" s="23"/>
-      <c r="E79" s="23"/>
-      <c r="F79" s="23"/>
-      <c r="G79" s="9">
-        <f>SUM(G66:G78)</f>
-        <v>1450500</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="21" t="s">
+      <c r="B82" s="21"/>
+      <c r="C82" s="21"/>
+      <c r="D82" s="21"/>
+      <c r="E82" s="21"/>
+      <c r="F82" s="21"/>
+      <c r="G82" s="9">
+        <f>SUM(G68:G81)</f>
+        <v>1479750</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A83" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="B80" s="21"/>
-      <c r="C80" s="21"/>
-      <c r="D80" s="21"/>
-      <c r="E80" s="21"/>
-      <c r="F80" s="21"/>
-      <c r="G80" s="21"/>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A81" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B81" s="2" t="s">
+      <c r="B83" s="23"/>
+      <c r="C83" s="23"/>
+      <c r="D83" s="23"/>
+      <c r="E83" s="23"/>
+      <c r="F83" s="23"/>
+      <c r="G83" s="23"/>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A84" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C81" s="3" t="s">
+      <c r="C84" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D81" s="3" t="s">
+      <c r="D84" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E81" s="3" t="s">
+      <c r="E84" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F81" s="4" t="s">
+      <c r="F84" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G81" s="4" t="s">
+      <c r="G84" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A82" s="5" t="s">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A85" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B82" s="6" t="s">
+      <c r="B85" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C82" s="7" t="s">
+      <c r="C85" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D82" s="7">
-        <v>3</v>
-      </c>
-      <c r="E82" s="7">
-        <v>3</v>
-      </c>
-      <c r="F82" s="8">
+      <c r="D85" s="7">
+        <v>3</v>
+      </c>
+      <c r="E85" s="7">
+        <v>3</v>
+      </c>
+      <c r="F85" s="8">
         <v>9000</v>
       </c>
-      <c r="G82" s="9">
-        <f>IF(OR(D82="",F82=""),0,D82*IF(E82="",1,E82)*F82)</f>
+      <c r="G85" s="9">
+        <f>IF(OR(D85="",F85=""),0,D85*IF(E85="",1,E85)*F85)</f>
         <v>81000</v>
       </c>
     </row>
-    <row r="83" spans="1:7" ht="22" x14ac:dyDescent="0.35">
-      <c r="A83" s="5" t="s">
+    <row r="86" spans="1:7" ht="22" x14ac:dyDescent="0.35">
+      <c r="A86" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B83" s="29" t="s">
+      <c r="B86" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="C83" s="7" t="s">
+      <c r="C86" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D83" s="7">
+      <c r="D86" s="7">
         <v>4</v>
       </c>
-      <c r="E83" s="7">
-        <v>3</v>
-      </c>
-      <c r="F83" s="8">
+      <c r="E86" s="7">
+        <v>3</v>
+      </c>
+      <c r="F86" s="8">
         <v>13500</v>
       </c>
-      <c r="G83" s="9">
-        <f>IF(OR(D83="",F83=""),0,D83*IF(E83="",1,E83)*F83)</f>
+      <c r="G86" s="9">
+        <f>IF(OR(D86="",F86=""),0,D86*IF(E86="",1,E86)*F86)</f>
         <v>162000</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A84" s="5" t="s">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A87" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B84" s="6" t="s">
+      <c r="B87" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C84" s="7" t="s">
+      <c r="C87" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="D84" s="7">
-        <v>1</v>
-      </c>
-      <c r="E84" s="7">
-        <v>3</v>
-      </c>
-      <c r="F84" s="8">
+      <c r="D87" s="7">
+        <v>1</v>
+      </c>
+      <c r="E87" s="7">
+        <v>3</v>
+      </c>
+      <c r="F87" s="8">
         <v>18000</v>
       </c>
-      <c r="G84" s="9">
-        <f>IF(OR(D84="",F84=""),0,D84*IF(E84="",1,E84)*F84)</f>
+      <c r="G87" s="9">
+        <f>IF(OR(D87="",F87=""),0,D87*IF(E87="",1,E87)*F87)</f>
         <v>54000</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A85" s="23" t="s">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A88" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="B85" s="23"/>
-      <c r="C85" s="23"/>
-      <c r="D85" s="23"/>
-      <c r="E85" s="23"/>
-      <c r="F85" s="23"/>
-      <c r="G85" s="10">
-        <f>SUM(G82:G84)</f>
+      <c r="B88" s="21"/>
+      <c r="C88" s="21"/>
+      <c r="D88" s="21"/>
+      <c r="E88" s="21"/>
+      <c r="F88" s="21"/>
+      <c r="G88" s="10">
+        <f>SUM(G85:G87)</f>
         <v>297000</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A86" s="23" t="s">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A89" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B86" s="23"/>
-      <c r="C86" s="23"/>
-      <c r="D86" s="23"/>
-      <c r="E86" s="23"/>
-      <c r="F86" s="23"/>
-      <c r="G86" s="10">
-        <f>SUM(G79,G85)</f>
-        <v>1747500</v>
+      <c r="B89" s="21"/>
+      <c r="C89" s="21"/>
+      <c r="D89" s="21"/>
+      <c r="E89" s="21"/>
+      <c r="F89" s="21"/>
+      <c r="G89" s="10">
+        <f>SUM(G82,G88)</f>
+        <v>1776750</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="A86:F86"/>
-    <mergeCell ref="A60:F60"/>
-    <mergeCell ref="A61:F61"/>
-    <mergeCell ref="A62:F62"/>
-    <mergeCell ref="A80:G80"/>
-    <mergeCell ref="A85:F85"/>
-    <mergeCell ref="A79:F79"/>
-    <mergeCell ref="A63:G63"/>
-    <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="A64:G64"/>
-    <mergeCell ref="A48:G48"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="A47:G47"/>
-    <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A38:F38"/>
+  <mergeCells count="30">
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="A7:G7"/>
     <mergeCell ref="A21:F21"/>
@@ -2901,6 +3016,27 @@
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A63:G64"/>
+    <mergeCell ref="A89:F89"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="A62:F62"/>
+    <mergeCell ref="A83:G83"/>
+    <mergeCell ref="A88:F88"/>
+    <mergeCell ref="A82:F82"/>
+    <mergeCell ref="A65:G65"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>